<commit_message>
Update all statstic files for September 2026
</commit_message>
<xml_diff>
--- a/statistics_files/2026/2026_99_y_graph.xlsx
+++ b/statistics_files/2026/2026_99_y_graph.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\George\Documents\github\next_statistics\statistics_files\2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Staff\Documents\GitHub\next_statistics\statistics_files\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8077D9-D75A-4AF5-A9BE-40DE8A68FD35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{404286D0-063D-48EE-8344-978B378A886A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1037,6 +1037,9 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>91059</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>90304</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2411,12 +2414,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2439,7 +2442,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2462,7 +2465,7 @@
         <v>86140</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2485,7 +2488,7 @@
         <v>81280</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2508,7 +2511,7 @@
         <v>88294</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2531,7 +2534,7 @@
         <v>79471</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -2554,7 +2557,7 @@
         <v>86748</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -2577,7 +2580,7 @@
         <v>108709</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -2600,7 +2603,7 @@
         <v>101271</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -2623,7 +2626,7 @@
         <v>91059</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2642,8 +2645,11 @@
       <c r="F10">
         <v>88575</v>
       </c>
+      <c r="G10">
+        <v>90304</v>
+      </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -2663,7 +2669,7 @@
         <v>90165</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -2683,7 +2689,7 @@
         <v>75089</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2703,7 +2709,7 @@
         <v>75089</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>13</v>
       </c>
@@ -2714,7 +2720,7 @@
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2723,7 +2729,7 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -2732,7 +2738,7 @@
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -2741,7 +2747,7 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2750,7 +2756,7 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -2759,7 +2765,7 @@
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -2768,7 +2774,7 @@
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -2777,7 +2783,7 @@
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -2786,7 +2792,7 @@
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -2795,7 +2801,7 @@
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -2804,7 +2810,7 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2813,7 +2819,7 @@
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -2822,7 +2828,7 @@
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -2831,7 +2837,7 @@
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>

</xml_diff>